<commit_message>
Correct indoor and outdoor LC60H reflective back MSRP to $888 for v1.70.5
</commit_message>
<xml_diff>
--- a/LocalData/pricing.xlsx
+++ b/LocalData/pricing.xlsx
@@ -17899,7 +17899,7 @@
         <x:v>732</x:v>
       </x:c>
       <x:c r="D244" s="4">
-        <x:v>799</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="E244" s="10"/>
     </x:row>
@@ -26926,7 +26926,7 @@
         <x:v>2164</x:v>
       </x:c>
       <x:c r="D109" s="35">
-        <x:v>799</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="E109" s="69"/>
     </x:row>

</xml_diff>

<commit_message>
Correct indoor and outdoor LC60H reflective back MSRP to $888 for v1.70.5 (#48)
</commit_message>
<xml_diff>
--- a/LocalData/pricing.xlsx
+++ b/LocalData/pricing.xlsx
@@ -17899,7 +17899,7 @@
         <x:v>732</x:v>
       </x:c>
       <x:c r="D244" s="4">
-        <x:v>799</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="E244" s="10"/>
     </x:row>
@@ -26926,7 +26926,7 @@
         <x:v>2164</x:v>
       </x:c>
       <x:c r="D109" s="35">
-        <x:v>799</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="E109" s="69"/>
     </x:row>

</xml_diff>